<commit_message>
Sync current local repository version
</commit_message>
<xml_diff>
--- a/02_APriori_PBPK_Workflow/Configurations/Scenarios.xlsx
+++ b/02_APriori_PBPK_Workflow/Configurations/Scenarios.xlsx
@@ -60,7 +60,7 @@
     <t xml:space="preserve">"Global", "Adalimumab_Human"</t>
   </si>
   <si>
-    <t xml:space="preserve">0, 12, 12; 12, 672, 0.1666667</t>
+    <t xml:space="preserve">0, 12, 12; 12, 2880, 0.1666667</t>
   </si>
   <si>
     <t xml:space="preserve">h</t>
@@ -614,7 +614,7 @@
     <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="52.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="28.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="29.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="30.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="18.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="15.71" hidden="0" customWidth="1"/>

</xml_diff>